<commit_message>
Update binary files for appointments and images
</commit_message>
<xml_diff>
--- a/excel-sheets/appointments.xlsx
+++ b/excel-sheets/appointments.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27932"/>
-  <workbookPr/>
+  <workbookPr hidePivotFieldList="1"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/39d657ef79bceff4/Desktop/colab/healthcare/excel-sheets/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2" documentId="8_{5C09FDDB-C570-4D60-86F0-45ABBAEFDFB7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AD624221-0ECB-432B-89E0-ED559B3A079E}"/>
+  <xr:revisionPtr revIDLastSave="13" documentId="8_{5C09FDDB-C570-4D60-86F0-45ABBAEFDFB7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7EC9EEBD-E4DD-4C44-BBE1-ACB517499933}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="683" firstSheet="2" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="683" firstSheet="2" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Raw Data" sheetId="1" r:id="rId1"/>
@@ -69,7 +69,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4661" uniqueCount="69">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4676" uniqueCount="69">
   <si>
     <t>patient_age</t>
   </si>
@@ -412,7 +412,1060 @@
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Percent" xfId="1" builtinId="5"/>
   </cellStyles>
-  <dxfs count="80">
+  <dxfs count="431">
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="166" formatCode="0.0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="166" formatCode="0.0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="166" formatCode="0.0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="166" formatCode="0.0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="166" formatCode="0.0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="166" formatCode="0.0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="166" formatCode="0.0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="166" formatCode="0.0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="166" formatCode="0.0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="166" formatCode="0.0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="166" formatCode="0.0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="166" formatCode="0.0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="166" formatCode="0.0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="166" formatCode="0.0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="166" formatCode="0.0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="166" formatCode="0.0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="166" formatCode="0.0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="166" formatCode="0.0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="166" formatCode="0.0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="166" formatCode="0.0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="166" formatCode="0.0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="166" formatCode="0.0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="166" formatCode="0.0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="166" formatCode="0.0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="166" formatCode="0.0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="166" formatCode="0.0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="166" formatCode="0.0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="166" formatCode="0.0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="166" formatCode="0.0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="166" formatCode="0.0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="166" formatCode="0.0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="166" formatCode="0.0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="166" formatCode="0.0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="166" formatCode="0.0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="166" formatCode="0.0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="166" formatCode="0.0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="166" formatCode="0.0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="166" formatCode="0.0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="166" formatCode="0.0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
     <dxf>
       <numFmt numFmtId="1" formatCode="0"/>
     </dxf>
@@ -1269,13 +2322,13 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="3"/>
                 <c:pt idx="0">
-                  <c:v>15</c:v>
+                  <c:v>101</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>63</c:v>
+                  <c:v>343</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>14</c:v>
+                  <c:v>56</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1761,28 +2814,28 @@
               <c:strCache>
                 <c:ptCount val="8"/>
                 <c:pt idx="0">
+                  <c:v>Mymensingh</c:v>
+                </c:pt>
+                <c:pt idx="1">
                   <c:v>Sylhet</c:v>
                 </c:pt>
-                <c:pt idx="1">
+                <c:pt idx="2">
                   <c:v>Rajshahi</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>Dhaka</c:v>
                 </c:pt>
                 <c:pt idx="3">
                   <c:v>Khulna</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>Barishal</c:v>
+                  <c:v>Dhaka</c:v>
                 </c:pt>
                 <c:pt idx="5">
                   <c:v>Chattogram</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>Rangpur</c:v>
+                  <c:v>Barishal</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>Mymensingh</c:v>
+                  <c:v>Rangpur</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -1794,28 +2847,28 @@
                 <c:formatCode>0.00</c:formatCode>
                 <c:ptCount val="8"/>
                 <c:pt idx="0">
-                  <c:v>11.5</c:v>
+                  <c:v>11.44</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>11.111111111111111</c:v>
+                  <c:v>11.348837209302326</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>10.071428571428571</c:v>
+                  <c:v>10.95</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>9.0833333333333339</c:v>
+                  <c:v>10.633333333333333</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>8.8000000000000007</c:v>
+                  <c:v>10.512658227848101</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>8.4642857142857135</c:v>
+                  <c:v>10.375</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>7.666666666666667</c:v>
+                  <c:v>9.2727272727272734</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>4.666666666666667</c:v>
+                  <c:v>7.7</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2476,23 +3529,53 @@
           </c:dLbls>
           <c:cat>
             <c:strRef>
-              <c:f>'Appointment Pivot Tables'!$G$9:$G$10</c:f>
+              <c:f>'Appointment Pivot Tables'!$G$9:$G$15</c:f>
               <c:strCache>
-                <c:ptCount val="1"/>
+                <c:ptCount val="6"/>
                 <c:pt idx="0">
+                  <c:v>General Physician</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Gynecologist</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Orthopedic</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>Dermatologist</c:v>
+                </c:pt>
+                <c:pt idx="4">
                   <c:v>Pediatrician</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>Cardiologist</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'Appointment Pivot Tables'!$H$9:$H$10</c:f>
+              <c:f>'Appointment Pivot Tables'!$H$9:$H$15</c:f>
               <c:numCache>
                 <c:formatCode>0.00</c:formatCode>
-                <c:ptCount val="1"/>
+                <c:ptCount val="6"/>
                 <c:pt idx="0">
+                  <c:v>11.55952380952381</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>11.546666666666667</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>11.48</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>10.49438202247191</c:v>
+                </c:pt>
+                <c:pt idx="4">
                   <c:v>9.2934782608695645</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>8.9764705882352942</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -3163,23 +4246,53 @@
           </c:dLbls>
           <c:cat>
             <c:strRef>
-              <c:f>'Appointment Pivot Tables'!$D$33:$D$34</c:f>
+              <c:f>'Appointment Pivot Tables'!$D$33:$D$39</c:f>
               <c:strCache>
-                <c:ptCount val="1"/>
+                <c:ptCount val="6"/>
                 <c:pt idx="0">
+                  <c:v>General Physician</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Dermatologist</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Gynecologist</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>Orthopedic</c:v>
+                </c:pt>
+                <c:pt idx="4">
                   <c:v>Pediatrician</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>Cardiologist</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'Appointment Pivot Tables'!$E$33:$E$34</c:f>
+              <c:f>'Appointment Pivot Tables'!$E$33:$E$39</c:f>
               <c:numCache>
                 <c:formatCode>0</c:formatCode>
-                <c:ptCount val="1"/>
+                <c:ptCount val="6"/>
                 <c:pt idx="0">
+                  <c:v>971</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>934</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>866</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>861</c:v>
+                </c:pt>
+                <c:pt idx="4">
                   <c:v>855</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>763</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -3891,16 +5004,16 @@
                 <c:formatCode>0.00</c:formatCode>
                 <c:ptCount val="4"/>
                 <c:pt idx="0">
-                  <c:v>10.75</c:v>
+                  <c:v>10.784615384615385</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>9.1304347826086953</c:v>
+                  <c:v>10.754237288135593</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>8.7741935483870961</c:v>
+                  <c:v>10.246913580246913</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>8.2142857142857135</c:v>
+                  <c:v>10.21111111111111</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -4600,16 +5713,16 @@
                 <c:formatCode>0</c:formatCode>
                 <c:ptCount val="4"/>
                 <c:pt idx="0">
-                  <c:v>272</c:v>
+                  <c:v>1660</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>258</c:v>
+                  <c:v>1402</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>210</c:v>
+                  <c:v>1269</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>115</c:v>
+                  <c:v>919</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -5284,28 +6397,28 @@
               <c:strCache>
                 <c:ptCount val="8"/>
                 <c:pt idx="0">
+                  <c:v>Dhaka</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Chattogram</c:v>
+                </c:pt>
+                <c:pt idx="2">
                   <c:v>Rajshahi</c:v>
                 </c:pt>
-                <c:pt idx="1">
-                  <c:v>Dhaka</c:v>
+                <c:pt idx="3">
+                  <c:v>Sylhet</c:v>
                 </c:pt>
-                <c:pt idx="2">
-                  <c:v>Chattogram</c:v>
+                <c:pt idx="4">
+                  <c:v>Mymensingh</c:v>
                 </c:pt>
-                <c:pt idx="3">
+                <c:pt idx="5">
                   <c:v>Khulna</c:v>
                 </c:pt>
-                <c:pt idx="4">
-                  <c:v>Sylhet</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>Rangpur</c:v>
-                </c:pt>
                 <c:pt idx="6">
-                  <c:v>Mymensingh</c:v>
+                  <c:v>Barishal</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>Barishal</c:v>
+                  <c:v>Rangpur</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -5317,25 +6430,25 @@
                 <c:formatCode>0.00%</c:formatCode>
                 <c:ptCount val="8"/>
                 <c:pt idx="0">
-                  <c:v>0.33333333333333331</c:v>
+                  <c:v>0.14556962025316456</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.25</c:v>
+                  <c:v>0.13392857142857142</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0.10714285714285714</c:v>
+                  <c:v>0.11666666666666667</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>8.3333333333333329E-2</c:v>
+                  <c:v>9.3023255813953487E-2</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0</c:v>
+                  <c:v>0.08</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>0</c:v>
+                  <c:v>6.6666666666666666E-2</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>0</c:v>
+                  <c:v>4.5454545454545456E-2</c:v>
                 </c:pt>
                 <c:pt idx="7">
                   <c:v>0</c:v>
@@ -6061,40 +7174,40 @@
                 <c:formatCode>0.00%</c:formatCode>
                 <c:ptCount val="12"/>
                 <c:pt idx="0">
-                  <c:v>0</c:v>
+                  <c:v>9.0909090909090912E-2</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.125</c:v>
+                  <c:v>0.13513513513513514</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0</c:v>
+                  <c:v>8.3333333333333329E-2</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.14285714285714285</c:v>
+                  <c:v>0.11764705882352941</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0.66666666666666663</c:v>
+                  <c:v>0.15</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>0.125</c:v>
+                  <c:v>8.5106382978723402E-2</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>0</c:v>
+                  <c:v>0.15789473684210525</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>0.125</c:v>
+                  <c:v>0.13513513513513514</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>0.375</c:v>
+                  <c:v>0.21621621621621623</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>0.14285714285714285</c:v>
+                  <c:v>6.3829787234042548E-2</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>0.25</c:v>
+                  <c:v>9.6153846153846159E-2</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>0.22222222222222221</c:v>
+                  <c:v>5.128205128205128E-2</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -6765,23 +7878,53 @@
           </c:dLbls>
           <c:cat>
             <c:strRef>
-              <c:f>'Appointment Pivot Tables'!$G$19:$G$20</c:f>
+              <c:f>'Appointment Pivot Tables'!$G$19:$G$25</c:f>
               <c:strCache>
-                <c:ptCount val="1"/>
+                <c:ptCount val="6"/>
                 <c:pt idx="0">
                   <c:v>Pediatrician</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Dermatologist</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>General Physician</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>Orthopedic</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>Cardiologist</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>Gynecologist</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'Appointment Pivot Tables'!$H$19:$H$20</c:f>
+              <c:f>'Appointment Pivot Tables'!$H$19:$H$25</c:f>
               <c:numCache>
                 <c:formatCode>0.00%</c:formatCode>
-                <c:ptCount val="1"/>
+                <c:ptCount val="6"/>
                 <c:pt idx="0">
                   <c:v>0.15217391304347827</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0.1348314606741573</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>0.10714285714285714</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>0.10666666666666667</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>0.10588235294117647</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>5.3333333333333337E-2</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -7442,10 +8585,10 @@
               <c:strCache>
                 <c:ptCount val="4"/>
                 <c:pt idx="0">
-                  <c:v>Senior (56+)</c:v>
+                  <c:v>Child (0-17)</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>Child (0-17)</c:v>
+                  <c:v>Senior (56+)</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>Middle Age (36-55)</c:v>
@@ -7463,16 +8606,16 @@
                 <c:formatCode>0.00%</c:formatCode>
                 <c:ptCount val="4"/>
                 <c:pt idx="0">
-                  <c:v>0.22580645161290322</c:v>
+                  <c:v>0.15555555555555556</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.21428571428571427</c:v>
+                  <c:v>0.1419753086419753</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0.125</c:v>
+                  <c:v>0.1076923076923077</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>4.3478260869565216E-2</c:v>
+                  <c:v>4.2372881355932202E-2</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -8241,40 +9384,40 @@
                 <c:formatCode>0</c:formatCode>
                 <c:ptCount val="12"/>
                 <c:pt idx="0">
-                  <c:v>9</c:v>
+                  <c:v>44</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>8</c:v>
+                  <c:v>37</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>10</c:v>
+                  <c:v>48</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>7</c:v>
+                  <c:v>34</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>3</c:v>
+                  <c:v>40</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>8</c:v>
+                  <c:v>47</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>7</c:v>
+                  <c:v>38</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>8</c:v>
+                  <c:v>37</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>8</c:v>
+                  <c:v>37</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>7</c:v>
+                  <c:v>47</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>8</c:v>
+                  <c:v>52</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>9</c:v>
+                  <c:v>39</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -8966,22 +10109,22 @@
                   <c:v>Chattogram</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>Khulna</c:v>
+                  <c:v>Rajshahi</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>Rajshahi</c:v>
+                  <c:v>Khulna</c:v>
                 </c:pt>
                 <c:pt idx="4">
                   <c:v>Sylhet</c:v>
                 </c:pt>
                 <c:pt idx="5">
+                  <c:v>Mymensingh</c:v>
+                </c:pt>
+                <c:pt idx="6">
                   <c:v>Barishal</c:v>
                 </c:pt>
-                <c:pt idx="6">
+                <c:pt idx="7">
                   <c:v>Rangpur</c:v>
-                </c:pt>
-                <c:pt idx="7">
-                  <c:v>Mymensingh</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -8993,28 +10136,28 @@
                 <c:formatCode>0</c:formatCode>
                 <c:ptCount val="8"/>
                 <c:pt idx="0">
-                  <c:v>282</c:v>
+                  <c:v>1661</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>237</c:v>
+                  <c:v>1162</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>109</c:v>
+                  <c:v>657</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>100</c:v>
+                  <c:v>638</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>46</c:v>
+                  <c:v>488</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>44</c:v>
+                  <c:v>286</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>23</c:v>
+                  <c:v>204</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>14</c:v>
+                  <c:v>154</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -9737,40 +10880,40 @@
                 <c:formatCode>0.00</c:formatCode>
                 <c:ptCount val="12"/>
                 <c:pt idx="0">
-                  <c:v>7.5555555555555554</c:v>
+                  <c:v>10.659090909090908</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>8.625</c:v>
+                  <c:v>10.567567567567568</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>11.8</c:v>
+                  <c:v>11.3125</c:v>
                 </c:pt>
                 <c:pt idx="3">
+                  <c:v>9.382352941176471</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>9.8000000000000007</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>12.212765957446809</c:v>
+                </c:pt>
+                <c:pt idx="6">
                   <c:v>9</c:v>
                 </c:pt>
-                <c:pt idx="4">
-                  <c:v>15.333333333333334</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>10.25</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>10</c:v>
-                </c:pt>
                 <c:pt idx="7">
-                  <c:v>10.625</c:v>
+                  <c:v>9.6486486486486491</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>6.625</c:v>
+                  <c:v>9.8378378378378386</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>6.8571428571428568</c:v>
+                  <c:v>10.148936170212766</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>10</c:v>
+                  <c:v>12.307692307692308</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>8.1111111111111107</c:v>
+                  <c:v>9.7948717948717956</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -10491,40 +11634,40 @@
                 <c:formatCode>0</c:formatCode>
                 <c:ptCount val="12"/>
                 <c:pt idx="0">
-                  <c:v>68</c:v>
+                  <c:v>469</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>69</c:v>
+                  <c:v>391</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>118</c:v>
+                  <c:v>543</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>63</c:v>
+                  <c:v>319</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>46</c:v>
+                  <c:v>392</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>82</c:v>
+                  <c:v>574</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>70</c:v>
+                  <c:v>342</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>85</c:v>
+                  <c:v>357</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>53</c:v>
+                  <c:v>364</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>48</c:v>
+                  <c:v>477</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>80</c:v>
+                  <c:v>640</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>73</c:v>
+                  <c:v>382</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -18913,14 +20056,14 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>7</xdr:col>
-      <xdr:colOff>83820</xdr:colOff>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>411480</xdr:colOff>
       <xdr:row>0</xdr:row>
       <xdr:rowOff>137160</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>16</xdr:col>
-      <xdr:colOff>236220</xdr:colOff>
+      <xdr:colOff>487680</xdr:colOff>
       <xdr:row>2</xdr:row>
       <xdr:rowOff>121920</xdr:rowOff>
     </xdr:to>
@@ -18937,8 +20080,8 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="4351020" y="137160"/>
-          <a:ext cx="5638800" cy="350520"/>
+          <a:off x="4069080" y="137160"/>
+          <a:ext cx="6172200" cy="350520"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -18972,7 +20115,7 @@
                 <a:schemeClr val="bg1"/>
               </a:solidFill>
             </a:rPr>
-            <a:t>Appointment No Show Analysis Dashboard</a:t>
+            <a:t>Appointment Volume and No-Show Dashboard</a:t>
           </a:r>
           <a:endParaRPr lang="en-US" sz="2400" b="1">
             <a:solidFill>
@@ -19826,7 +20969,7 @@
                 <a:cs typeface="Calibri"/>
               </a:rPr>
               <a:pPr algn="ctr"/>
-              <a:t>92</a:t>
+              <a:t>500</a:t>
             </a:fld>
             <a:endParaRPr lang="en-US" sz="2000" b="1">
               <a:solidFill>
@@ -19998,7 +21141,7 @@
                 <a:cs typeface="Calibri"/>
               </a:rPr>
               <a:pPr algn="ctr"/>
-              <a:t>14</a:t>
+              <a:t>56</a:t>
             </a:fld>
             <a:endParaRPr lang="en-US" sz="2000" b="1">
               <a:solidFill>
@@ -20168,7 +21311,7 @@
                 <a:cs typeface="Calibri"/>
               </a:rPr>
               <a:pPr algn="ctr"/>
-              <a:t>15.2%</a:t>
+              <a:t>11.2%</a:t>
             </a:fld>
             <a:endParaRPr lang="en-US" sz="2000" b="1">
               <a:solidFill>
@@ -20753,16 +21896,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>6</xdr:col>
-      <xdr:colOff>281940</xdr:colOff>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>579120</xdr:colOff>
       <xdr:row>0</xdr:row>
-      <xdr:rowOff>38100</xdr:rowOff>
+      <xdr:rowOff>53340</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>16</xdr:col>
-      <xdr:colOff>106680</xdr:colOff>
+      <xdr:col>17</xdr:col>
+      <xdr:colOff>403860</xdr:colOff>
       <xdr:row>2</xdr:row>
-      <xdr:rowOff>22860</xdr:rowOff>
+      <xdr:rowOff>38100</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
@@ -20777,7 +21920,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="3939540" y="38100"/>
+          <a:off x="4846320" y="53340"/>
           <a:ext cx="5920740" cy="350520"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -20812,7 +21955,7 @@
                 <a:schemeClr val="bg1"/>
               </a:solidFill>
             </a:rPr>
-            <a:t>Appointment Wait Days Analysis Dashboard</a:t>
+            <a:t>Appointment Wait Days Dashboard</a:t>
           </a:r>
           <a:endParaRPr lang="en-US" sz="2400" b="1">
             <a:solidFill>
@@ -21031,7 +22174,7 @@
                 <a:cs typeface="Calibri"/>
               </a:rPr>
               <a:pPr algn="ctr"/>
-              <a:t>9.3</a:t>
+              <a:t>10.5</a:t>
             </a:fld>
             <a:endParaRPr lang="en-US" sz="2000" b="1">
               <a:solidFill>
@@ -21203,7 +22346,7 @@
                 <a:cs typeface="Calibri"/>
               </a:rPr>
               <a:pPr algn="ctr"/>
-              <a:t>855</a:t>
+              <a:t>5250</a:t>
             </a:fld>
             <a:endParaRPr lang="en-US" sz="2000" b="1">
               <a:solidFill>
@@ -29351,11 +30494,11 @@
     </pivotField>
     <pivotField showAll="0">
       <items count="7">
-        <item h="1" x="1"/>
-        <item h="1" x="5"/>
-        <item h="1" x="4"/>
-        <item h="1" x="0"/>
-        <item h="1" x="3"/>
+        <item x="1"/>
+        <item x="5"/>
+        <item x="4"/>
+        <item x="0"/>
+        <item x="3"/>
         <item x="2"/>
         <item t="default"/>
       </items>
@@ -29788,13 +30931,13 @@
     <dataField name="Average of Wait Days" fld="6" subtotal="average" baseField="0" baseItem="0" numFmtId="166"/>
   </dataFields>
   <formats count="1">
-    <format dxfId="71">
+    <format dxfId="422">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
   </formats>
   <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
   <filters count="1">
-    <filter fld="7" type="dateBetween" evalOrder="-1" id="1551" name="Appointment Date">
+    <filter fld="7" type="dateBetween" evalOrder="-1" id="1614" name="Appointment Date">
       <autoFilter ref="A1">
         <filterColumn colId="0">
           <customFilters and="1">
@@ -29848,11 +30991,11 @@
     </pivotField>
     <pivotField showAll="0">
       <items count="7">
-        <item h="1" x="1"/>
-        <item h="1" x="5"/>
-        <item h="1" x="4"/>
-        <item h="1" x="0"/>
-        <item h="1" x="3"/>
+        <item x="1"/>
+        <item x="5"/>
+        <item x="4"/>
+        <item x="0"/>
+        <item x="3"/>
         <item x="2"/>
         <item t="default"/>
       </items>
@@ -30338,7 +31481,7 @@
   </chartFormats>
   <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
   <filters count="1">
-    <filter fld="7" type="dateBetween" evalOrder="-1" id="1551" name="Appointment Date">
+    <filter fld="7" type="dateBetween" evalOrder="-1" id="1614" name="Appointment Date">
       <autoFilter ref="A1">
         <filterColumn colId="0">
           <customFilters and="1">
@@ -30392,11 +31535,11 @@
     </pivotField>
     <pivotField showAll="0">
       <items count="7">
-        <item h="1" x="1"/>
-        <item h="1" x="5"/>
-        <item h="1" x="4"/>
-        <item h="1" x="0"/>
-        <item h="1" x="3"/>
+        <item x="1"/>
+        <item x="5"/>
+        <item x="4"/>
+        <item x="0"/>
+        <item x="3"/>
         <item x="2"/>
         <item t="default"/>
       </items>
@@ -30830,7 +31973,7 @@
   </dataFields>
   <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
   <filters count="1">
-    <filter fld="7" type="dateBetween" evalOrder="-1" id="1551" name="Appointment Date">
+    <filter fld="7" type="dateBetween" evalOrder="-1" id="1614" name="Appointment Date">
       <autoFilter ref="A1">
         <filterColumn colId="0">
           <customFilters and="1">
@@ -30893,11 +32036,11 @@
     </pivotField>
     <pivotField showAll="0">
       <items count="7">
-        <item h="1" x="1"/>
-        <item h="1" x="5"/>
-        <item h="1" x="4"/>
-        <item h="1" x="0"/>
-        <item h="1" x="3"/>
+        <item x="1"/>
+        <item x="5"/>
+        <item x="4"/>
+        <item x="0"/>
+        <item x="3"/>
         <item x="2"/>
         <item t="default"/>
       </items>
@@ -31331,22 +32474,22 @@
       <x v="1"/>
     </i>
     <i>
+      <x v="5"/>
+    </i>
+    <i>
       <x v="3"/>
     </i>
     <i>
-      <x v="5"/>
+      <x v="7"/>
     </i>
     <i>
-      <x v="7"/>
+      <x v="4"/>
     </i>
     <i>
       <x/>
     </i>
     <i>
       <x v="6"/>
-    </i>
-    <i>
-      <x v="4"/>
     </i>
     <i t="grand">
       <x/>
@@ -31371,7 +32514,7 @@
   </chartFormats>
   <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
   <filters count="1">
-    <filter fld="7" type="dateBetween" evalOrder="-1" id="1551" name="Appointment Date">
+    <filter fld="7" type="dateBetween" evalOrder="-1" id="1614" name="Appointment Date">
       <autoFilter ref="A1">
         <filterColumn colId="0">
           <customFilters and="1">
@@ -31400,7 +32543,7 @@
 
 <file path=xl/pivotTables/pivotTable13.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{1815C2BF-B998-4588-A95C-906C88DA91E4}" name="PT12_Specialty_Average_Wait_Days" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="5" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="6" rowHeaderCaption="Specialty">
-  <location ref="G8:H10" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
+  <location ref="G8:H15" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="15">
     <pivotField showAll="0"/>
     <pivotField showAll="0">
@@ -31425,11 +32568,11 @@
     </pivotField>
     <pivotField axis="axisRow" showAll="0" sortType="descending">
       <items count="7">
-        <item h="1" x="1"/>
-        <item h="1" x="5"/>
-        <item h="1" x="4"/>
-        <item h="1" x="0"/>
-        <item h="1" x="3"/>
+        <item x="1"/>
+        <item x="5"/>
+        <item x="4"/>
+        <item x="0"/>
+        <item x="3"/>
         <item x="2"/>
         <item t="default"/>
       </items>
@@ -31864,9 +33007,24 @@
   <rowFields count="1">
     <field x="3"/>
   </rowFields>
-  <rowItems count="2">
+  <rowItems count="7">
+    <i>
+      <x v="2"/>
+    </i>
+    <i>
+      <x v="3"/>
+    </i>
+    <i>
+      <x v="4"/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
     <i>
       <x v="5"/>
+    </i>
+    <i>
+      <x/>
     </i>
     <i t="grand">
       <x/>
@@ -31900,7 +33058,7 @@
   </chartFormats>
   <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
   <filters count="1">
-    <filter fld="7" type="dateBetween" evalOrder="-1" id="1551" name="Appointment Date">
+    <filter fld="7" type="dateBetween" evalOrder="-1" id="1614" name="Appointment Date">
       <autoFilter ref="A1">
         <filterColumn colId="0">
           <customFilters and="1">
@@ -31954,11 +33112,11 @@
     </pivotField>
     <pivotField showAll="0">
       <items count="7">
-        <item h="1" x="1"/>
-        <item h="1" x="5"/>
-        <item h="1" x="4"/>
-        <item h="1" x="0"/>
-        <item h="1" x="3"/>
+        <item x="1"/>
+        <item x="5"/>
+        <item x="4"/>
+        <item x="0"/>
+        <item x="3"/>
         <item x="2"/>
         <item t="default"/>
       </items>
@@ -32392,7 +33550,7 @@
   </dataFields>
   <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
   <filters count="1">
-    <filter fld="7" type="dateBetween" evalOrder="-1" id="1551" name="Appointment Date">
+    <filter fld="7" type="dateBetween" evalOrder="-1" id="1614" name="Appointment Date">
       <autoFilter ref="A1">
         <filterColumn colId="0">
           <customFilters and="1">
@@ -32446,11 +33604,11 @@
     </pivotField>
     <pivotField showAll="0">
       <items count="7">
-        <item h="1" x="1"/>
-        <item h="1" x="5"/>
-        <item h="1" x="4"/>
-        <item h="1" x="0"/>
-        <item h="1" x="3"/>
+        <item x="1"/>
+        <item x="5"/>
+        <item x="4"/>
+        <item x="0"/>
+        <item x="3"/>
         <item x="2"/>
         <item t="default"/>
       </items>
@@ -32894,7 +34052,7 @@
   </dataFields>
   <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
   <filters count="1">
-    <filter fld="7" type="dateBetween" evalOrder="-1" id="1551" name="Appointment Date">
+    <filter fld="7" type="dateBetween" evalOrder="-1" id="1614" name="Appointment Date">
       <autoFilter ref="A1">
         <filterColumn colId="0">
           <customFilters and="1">
@@ -32923,7 +34081,7 @@
 
 <file path=xl/pivotTables/pivotTable16.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{508C7D23-63B7-4DD7-BBB8-38BA79153887}" name="PT19_Specialty_Sum_Wait_Days" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="5" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="4" rowHeaderCaption="Specialty">
-  <location ref="D32:E34" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
+  <location ref="D32:E39" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="15">
     <pivotField showAll="0"/>
     <pivotField showAll="0">
@@ -32948,11 +34106,11 @@
     </pivotField>
     <pivotField axis="axisRow" showAll="0" sortType="descending">
       <items count="7">
-        <item h="1" x="1"/>
-        <item h="1" x="5"/>
-        <item h="1" x="4"/>
-        <item h="1" x="0"/>
-        <item h="1" x="3"/>
+        <item x="1"/>
+        <item x="5"/>
+        <item x="4"/>
+        <item x="0"/>
+        <item x="3"/>
         <item x="2"/>
         <item t="default"/>
       </items>
@@ -33387,9 +34545,24 @@
   <rowFields count="1">
     <field x="3"/>
   </rowFields>
-  <rowItems count="2">
+  <rowItems count="7">
+    <i>
+      <x v="2"/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i>
+      <x v="3"/>
+    </i>
+    <i>
+      <x v="4"/>
+    </i>
     <i>
       <x v="5"/>
+    </i>
+    <i>
+      <x/>
     </i>
     <i t="grand">
       <x/>
@@ -33432,7 +34605,7 @@
   </chartFormats>
   <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
   <filters count="1">
-    <filter fld="7" type="dateBetween" evalOrder="-1" id="1551" name="Appointment Date">
+    <filter fld="7" type="dateBetween" evalOrder="-1" id="1614" name="Appointment Date">
       <autoFilter ref="A1">
         <filterColumn colId="0">
           <customFilters and="1">
@@ -33486,11 +34659,11 @@
     </pivotField>
     <pivotField showAll="0">
       <items count="7">
-        <item h="1" x="1"/>
-        <item h="1" x="5"/>
-        <item h="1" x="4"/>
-        <item h="1" x="0"/>
-        <item h="1" x="3"/>
+        <item x="1"/>
+        <item x="5"/>
+        <item x="4"/>
+        <item x="0"/>
+        <item x="3"/>
         <item x="2"/>
         <item t="default"/>
       </items>
@@ -33976,7 +35149,7 @@
   </chartFormats>
   <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
   <filters count="1">
-    <filter fld="7" type="dateBetween" evalOrder="-1" id="1551" name="Appointment Date">
+    <filter fld="7" type="dateBetween" evalOrder="-1" id="1614" name="Appointment Date">
       <autoFilter ref="A1">
         <filterColumn colId="0">
           <customFilters and="1">
@@ -34030,11 +35203,11 @@
     </pivotField>
     <pivotField showAll="0" sortType="descending">
       <items count="7">
-        <item h="1" x="1"/>
-        <item h="1" x="5"/>
-        <item h="1" x="4"/>
-        <item h="1" x="0"/>
-        <item h="1" x="3"/>
+        <item x="1"/>
+        <item x="5"/>
+        <item x="4"/>
+        <item x="0"/>
+        <item x="3"/>
         <item x="2"/>
         <item t="default"/>
       </items>
@@ -34502,7 +35675,7 @@
     <dataField name="Sum of Wait Days" fld="6" baseField="8" baseItem="1" numFmtId="1"/>
   </dataFields>
   <formats count="1">
-    <format dxfId="78">
+    <format dxfId="429">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
   </formats>
@@ -34537,7 +35710,7 @@
   </chartFormats>
   <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
   <filters count="1">
-    <filter fld="7" type="dateBetween" evalOrder="-1" id="1551" name="Appointment Date">
+    <filter fld="7" type="dateBetween" evalOrder="-1" id="1614" name="Appointment Date">
       <autoFilter ref="A1">
         <filterColumn colId="0">
           <customFilters and="1">
@@ -34591,11 +35764,11 @@
     </pivotField>
     <pivotField showAll="0">
       <items count="7">
-        <item h="1" x="1"/>
-        <item h="1" x="5"/>
-        <item h="1" x="4"/>
-        <item h="1" x="0"/>
-        <item h="1" x="3"/>
+        <item x="1"/>
+        <item x="5"/>
+        <item x="4"/>
+        <item x="0"/>
+        <item x="3"/>
         <item x="2"/>
         <item t="default"/>
       </items>
@@ -35029,7 +36202,7 @@
   </dataFields>
   <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
   <filters count="1">
-    <filter fld="7" type="dateBetween" evalOrder="-1" id="1551" name="Appointment Date">
+    <filter fld="7" type="dateBetween" evalOrder="-1" id="1614" name="Appointment Date">
       <autoFilter ref="A1">
         <filterColumn colId="0">
           <customFilters and="1">
@@ -35092,11 +36265,11 @@
     </pivotField>
     <pivotField showAll="0">
       <items count="7">
-        <item h="1" x="1"/>
-        <item h="1" x="5"/>
-        <item h="1" x="4"/>
-        <item h="1" x="0"/>
-        <item h="1" x="3"/>
+        <item x="1"/>
+        <item x="5"/>
+        <item x="4"/>
+        <item x="0"/>
+        <item x="3"/>
         <item x="2"/>
         <item t="default"/>
       </items>
@@ -35524,28 +36697,28 @@
   </rowFields>
   <rowItems count="9">
     <i>
+      <x v="4"/>
+    </i>
+    <i>
       <x v="7"/>
     </i>
     <i>
       <x v="5"/>
     </i>
     <i>
+      <x v="3"/>
+    </i>
+    <i>
       <x v="2"/>
     </i>
     <i>
-      <x v="3"/>
+      <x v="1"/>
     </i>
     <i>
       <x/>
     </i>
     <i>
-      <x v="1"/>
-    </i>
-    <i>
       <x v="6"/>
-    </i>
-    <i>
-      <x v="4"/>
     </i>
     <i t="grand">
       <x/>
@@ -35579,7 +36752,7 @@
   </chartFormats>
   <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
   <filters count="1">
-    <filter fld="7" type="dateBetween" evalOrder="-1" id="1551" name="Appointment Date">
+    <filter fld="7" type="dateBetween" evalOrder="-1" id="1614" name="Appointment Date">
       <autoFilter ref="A1">
         <filterColumn colId="0">
           <customFilters and="1">
@@ -35608,7 +36781,7 @@
 
 <file path=xl/pivotTables/pivotTable20.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{3F906D27-1A1F-43F0-BC6D-05BF4E7DC828}" name="PT26_Specialty_Rate_No_Show" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="5" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="4" rowHeaderCaption="Specialty">
-  <location ref="G18:H20" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
+  <location ref="G18:H25" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="15">
     <pivotField showAll="0"/>
     <pivotField showAll="0">
@@ -35633,11 +36806,11 @@
     </pivotField>
     <pivotField axis="axisRow" showAll="0" sortType="descending">
       <items count="7">
-        <item h="1" x="1"/>
-        <item h="1" x="5"/>
-        <item h="1" x="4"/>
-        <item h="1" x="0"/>
-        <item h="1" x="3"/>
+        <item x="1"/>
+        <item x="5"/>
+        <item x="4"/>
+        <item x="0"/>
+        <item x="3"/>
         <item x="2"/>
         <item t="default"/>
       </items>
@@ -36072,9 +37245,24 @@
   <rowFields count="1">
     <field x="3"/>
   </rowFields>
-  <rowItems count="2">
+  <rowItems count="7">
     <i>
       <x v="5"/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i>
+      <x v="2"/>
+    </i>
+    <i>
+      <x v="4"/>
+    </i>
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="3"/>
     </i>
     <i t="grand">
       <x/>
@@ -36087,7 +37275,7 @@
     <dataField name="Rate of No Show " fld="11" subtotal="average" baseField="3" baseItem="5" numFmtId="10"/>
   </dataFields>
   <formats count="1">
-    <format dxfId="79">
+    <format dxfId="430">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
   </formats>
@@ -36122,7 +37310,7 @@
   </chartFormats>
   <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
   <filters count="1">
-    <filter fld="7" type="dateBetween" evalOrder="-1" id="1551" name="Appointment Date">
+    <filter fld="7" type="dateBetween" evalOrder="-1" id="1614" name="Appointment Date">
       <autoFilter ref="A1">
         <filterColumn colId="0">
           <customFilters and="1">
@@ -36176,11 +37364,11 @@
     </pivotField>
     <pivotField showAll="0">
       <items count="7">
-        <item h="1" x="1"/>
-        <item h="1" x="5"/>
-        <item h="1" x="4"/>
-        <item h="1" x="0"/>
-        <item h="1" x="3"/>
+        <item x="1"/>
+        <item x="5"/>
+        <item x="4"/>
+        <item x="0"/>
+        <item x="3"/>
         <item x="2"/>
         <item t="default"/>
       </items>
@@ -36682,7 +37870,7 @@
   </chartFormats>
   <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
   <filters count="1">
-    <filter fld="7" type="dateBetween" evalOrder="-1" id="1551" name="Appointment Date">
+    <filter fld="7" type="dateBetween" evalOrder="-1" id="1614" name="Appointment Date">
       <autoFilter ref="A1">
         <filterColumn colId="0">
           <customFilters and="1">
@@ -36745,11 +37933,11 @@
     </pivotField>
     <pivotField showAll="0">
       <items count="7">
-        <item h="1" x="1"/>
-        <item h="1" x="5"/>
-        <item h="1" x="4"/>
-        <item h="1" x="0"/>
-        <item h="1" x="3"/>
+        <item x="1"/>
+        <item x="5"/>
+        <item x="4"/>
+        <item x="0"/>
+        <item x="3"/>
         <item x="2"/>
         <item t="default"/>
       </items>
@@ -37177,28 +38365,28 @@
   </rowFields>
   <rowItems count="9">
     <i>
-      <x v="5"/>
-    </i>
-    <i>
       <x v="2"/>
     </i>
     <i>
       <x v="1"/>
     </i>
     <i>
-      <x v="3"/>
+      <x v="5"/>
     </i>
     <i>
       <x v="7"/>
     </i>
     <i>
-      <x v="6"/>
-    </i>
-    <i>
       <x v="4"/>
     </i>
     <i>
+      <x v="3"/>
+    </i>
+    <i>
       <x/>
+    </i>
+    <i>
+      <x v="6"/>
     </i>
     <i t="grand">
       <x/>
@@ -37211,14 +38399,14 @@
     <dataField name="Rate of No Show" fld="11" subtotal="average" baseField="2" baseItem="2" numFmtId="10"/>
   </dataFields>
   <formats count="2">
-    <format dxfId="73">
+    <format dxfId="424">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="1">
           <reference field="2" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="72">
+    <format dxfId="423">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
   </formats>
@@ -37244,7 +38432,7 @@
   </chartFormats>
   <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
   <filters count="1">
-    <filter fld="7" type="dateBetween" evalOrder="-1" id="1551" name="Appointment Date">
+    <filter fld="7" type="dateBetween" evalOrder="-1" id="1614" name="Appointment Date">
       <autoFilter ref="A1">
         <filterColumn colId="0">
           <customFilters and="1">
@@ -37298,11 +38486,11 @@
     </pivotField>
     <pivotField showAll="0">
       <items count="7">
-        <item h="1" x="1"/>
-        <item h="1" x="5"/>
-        <item h="1" x="4"/>
-        <item h="1" x="0"/>
-        <item h="1" x="3"/>
+        <item x="1"/>
+        <item x="5"/>
+        <item x="4"/>
+        <item x="0"/>
+        <item x="3"/>
         <item x="2"/>
         <item t="default"/>
       </items>
@@ -37736,7 +38924,7 @@
   </dataFields>
   <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
   <filters count="1">
-    <filter fld="7" type="dateBetween" evalOrder="-1" id="1551" name="Appointment Date">
+    <filter fld="7" type="dateBetween" evalOrder="-1" id="1614" name="Appointment Date">
       <autoFilter ref="A1">
         <filterColumn colId="0">
           <customFilters and="1">
@@ -37790,11 +38978,11 @@
     </pivotField>
     <pivotField showAll="0" sortType="descending">
       <items count="7">
-        <item h="1" x="1"/>
-        <item h="1" x="5"/>
-        <item h="1" x="4"/>
-        <item h="1" x="0"/>
-        <item h="1" x="3"/>
+        <item x="1"/>
+        <item x="5"/>
+        <item x="4"/>
+        <item x="0"/>
+        <item x="3"/>
         <item x="2"/>
         <item t="default"/>
       </items>
@@ -38277,7 +39465,7 @@
     <dataField name="Rate of No Show " fld="11" subtotal="average" baseField="0" baseItem="0" numFmtId="10"/>
   </dataFields>
   <formats count="1">
-    <format dxfId="74">
+    <format dxfId="425">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
   </formats>
@@ -38312,7 +39500,7 @@
   </chartFormats>
   <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
   <filters count="1">
-    <filter fld="7" type="dateBetween" evalOrder="-1" id="1551" name="Appointment Date">
+    <filter fld="7" type="dateBetween" evalOrder="-1" id="1614" name="Appointment Date">
       <autoFilter ref="A1">
         <filterColumn colId="0">
           <customFilters and="1">
@@ -38366,11 +39554,11 @@
     </pivotField>
     <pivotField showAll="0" sortType="descending">
       <items count="7">
-        <item h="1" x="1"/>
-        <item h="1" x="5"/>
-        <item h="1" x="4"/>
-        <item h="1" x="0"/>
-        <item h="1" x="3"/>
+        <item x="1"/>
+        <item x="5"/>
+        <item x="4"/>
+        <item x="0"/>
+        <item x="3"/>
         <item x="2"/>
         <item t="default"/>
       </items>
@@ -38816,10 +40004,10 @@
   </rowFields>
   <rowItems count="5">
     <i>
-      <x v="1"/>
+      <x v="3"/>
     </i>
     <i>
-      <x v="3"/>
+      <x v="1"/>
     </i>
     <i>
       <x v="2"/>
@@ -38838,7 +40026,7 @@
     <dataField name="Rate of No Show " fld="11" subtotal="average" baseField="3" baseItem="5" numFmtId="10"/>
   </dataFields>
   <formats count="1">
-    <format dxfId="75">
+    <format dxfId="426">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
   </formats>
@@ -38882,7 +40070,7 @@
   </chartFormats>
   <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
   <filters count="1">
-    <filter fld="7" type="dateBetween" evalOrder="-1" id="1551" name="Appointment Date">
+    <filter fld="7" type="dateBetween" evalOrder="-1" id="1614" name="Appointment Date">
       <autoFilter ref="A1">
         <filterColumn colId="0">
           <customFilters and="1">
@@ -38936,11 +40124,11 @@
     </pivotField>
     <pivotField showAll="0" sortType="descending">
       <items count="7">
-        <item h="1" x="1"/>
-        <item h="1" x="5"/>
-        <item h="1" x="4"/>
-        <item h="1" x="0"/>
-        <item h="1" x="3"/>
+        <item x="1"/>
+        <item x="5"/>
+        <item x="4"/>
+        <item x="0"/>
+        <item x="3"/>
         <item x="2"/>
         <item t="default"/>
       </items>
@@ -39438,7 +40626,7 @@
   </chartFormats>
   <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
   <filters count="1">
-    <filter fld="7" type="dateBetween" evalOrder="-1" id="1551" name="Appointment Date">
+    <filter fld="7" type="dateBetween" evalOrder="-1" id="1614" name="Appointment Date">
       <autoFilter ref="A1">
         <filterColumn colId="0">
           <customFilters and="1">
@@ -39492,11 +40680,11 @@
     </pivotField>
     <pivotField showAll="0">
       <items count="7">
-        <item h="1" x="1"/>
-        <item h="1" x="5"/>
-        <item h="1" x="4"/>
-        <item h="1" x="0"/>
-        <item h="1" x="3"/>
+        <item x="1"/>
+        <item x="5"/>
+        <item x="4"/>
+        <item x="0"/>
+        <item x="3"/>
         <item x="2"/>
         <item t="default"/>
       </items>
@@ -39970,10 +41158,10 @@
     <dataField name="Total Appointments" fld="2" subtotal="count" baseField="0" baseItem="0" numFmtId="1"/>
   </dataFields>
   <formats count="2">
-    <format dxfId="77">
+    <format dxfId="428">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
-    <format dxfId="76">
+    <format dxfId="427">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" axis="axisValues" fieldPosition="0"/>
     </format>
   </formats>
@@ -39999,7 +41187,7 @@
   </chartFormats>
   <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
   <filters count="1">
-    <filter fld="7" type="dateBetween" evalOrder="-1" id="1551" name="Appointment Date">
+    <filter fld="7" type="dateBetween" evalOrder="-1" id="1614" name="Appointment Date">
       <autoFilter ref="A1">
         <filterColumn colId="0">
           <customFilters and="1">
@@ -40129,11 +41317,11 @@
   <data>
     <tabular pivotCacheId="2030443388">
       <items count="6">
-        <i x="1"/>
-        <i x="5"/>
-        <i x="4"/>
-        <i x="0"/>
-        <i x="3"/>
+        <i x="1" s="1"/>
+        <i x="5" s="1"/>
+        <i x="4" s="1"/>
+        <i x="0" s="1"/>
+        <i x="3" s="1"/>
         <i x="2" s="1"/>
       </items>
     </tabular>
@@ -40188,10 +41376,10 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{3F0A18D8-50A1-40C2-A2A8-FF9A745DC306}" name="Table2" displayName="Table2" ref="F3:F4" totalsRowShown="0" headerRowDxfId="70" dataDxfId="69" dataCellStyle="Percent">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{3F0A18D8-50A1-40C2-A2A8-FF9A745DC306}" name="Table2" displayName="Table2" ref="F3:F4" totalsRowShown="0" headerRowDxfId="421" dataDxfId="420" dataCellStyle="Percent">
   <autoFilter ref="F3:F4" xr:uid="{3F0A18D8-50A1-40C2-A2A8-FF9A745DC306}"/>
   <tableColumns count="1">
-    <tableColumn id="1" xr3:uid="{C5576054-70BB-44F5-8FAF-3AEF21F8A9B4}" name="No-Show Percentage" dataDxfId="68" dataCellStyle="Percent">
+    <tableColumn id="1" xr3:uid="{C5576054-70BB-44F5-8FAF-3AEF21F8A9B4}" name="No-Show Percentage" dataDxfId="419" dataCellStyle="Percent">
       <calculatedColumnFormula>(C4/A4)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -40200,7 +41388,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{38F03D7D-02C0-4D42-99AE-645D69A22E56}" name="Bangladesh_Appointment_Trends" displayName="Bangladesh_Appointment_Trends" ref="A1:L501" totalsRowShown="0" headerRowDxfId="67" headerRowBorderDxfId="66" tableBorderDxfId="65">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{38F03D7D-02C0-4D42-99AE-645D69A22E56}" name="Bangladesh_Appointment_Trends" displayName="Bangladesh_Appointment_Trends" ref="A1:L501" totalsRowShown="0" headerRowDxfId="418" headerRowBorderDxfId="417" tableBorderDxfId="416">
   <autoFilter ref="A1:L501" xr:uid="{38F03D7D-02C0-4D42-99AE-645D69A22E56}"/>
   <tableColumns count="12">
     <tableColumn id="1" xr3:uid="{CCFC8FA1-CFD0-4FE7-8136-B21D5FC0AECC}" name="Age"/>
@@ -40210,7 +41398,7 @@
     <tableColumn id="5" xr3:uid="{22CCBC37-AE6B-4E66-B591-4E37EE42920B}" name="Appointment Status"/>
     <tableColumn id="6" xr3:uid="{5AE11F70-F6F6-4154-AC12-6A9E8C61D300}" name="Consultation Fee"/>
     <tableColumn id="7" xr3:uid="{B0A9B937-A8C7-4586-8A68-F863E459A39F}" name="Wait Days"/>
-    <tableColumn id="8" xr3:uid="{77C6BDDE-7D1A-4120-91E3-DFD366A69F8C}" name="Appointment Date" dataDxfId="64"/>
+    <tableColumn id="8" xr3:uid="{77C6BDDE-7D1A-4120-91E3-DFD366A69F8C}" name="Appointment Date" dataDxfId="415"/>
     <tableColumn id="9" xr3:uid="{51CD8388-E175-4F42-B96E-F5820AD156F1}" name="Age Group"/>
     <tableColumn id="10" xr3:uid="{DEBAF746-ED9A-4CC1-8E78-EA0A422026E0}" name="Day of Week">
       <calculatedColumnFormula>TEXT(H2,"dddd")</calculatedColumnFormula>
@@ -40218,7 +41406,7 @@
     <tableColumn id="11" xr3:uid="{CC8125A2-0D24-4E4F-80B7-7DC184465B70}" name="Day Type">
       <calculatedColumnFormula>IF(WEEKDAY(H2,1)&gt;5,"Weekend","Weekday")</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="12" xr3:uid="{1298B857-864D-4AE2-BBF3-90B94A9CF7AA}" name="No Show Flag" dataDxfId="63">
+    <tableColumn id="12" xr3:uid="{1298B857-864D-4AE2-BBF3-90B94A9CF7AA}" name="No Show Flag" dataDxfId="414">
       <calculatedColumnFormula>IF(Bangladesh_Appointment_Trends[[#This Row],[Appointment Status]]="No-Show",1,0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -40544,8 +41732,8 @@
 <timelines xmlns="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" mc:Ignorable="x xr10">
   <timeline name="Appointment Date" xr10:uid="{BB2F94B3-43A2-44D5-9ECC-2F3B81B725B6}" cache="NativeTimeline_Appointment_Date" caption="Year" level="0" selectionLevel="0" scrollPosition="2023-01-01T00:00:00"/>
   <timeline name="Appointment Date 1" xr10:uid="{D794BFE3-4BF9-4A1A-902C-3B6EF0DC755F}" cache="NativeTimeline_Appointment_Date" caption="Quarter" level="1" selectionLevel="0" scrollPosition="2023-01-01T00:00:00"/>
-  <timeline name="Appointment Date 2" xr10:uid="{527740AB-750D-4187-8225-16D51394F21D}" cache="NativeTimeline_Appointment_Date" caption="Month" level="2" selectionLevel="0" scrollPosition="2023-03-11T00:00:00"/>
-  <timeline name="Appointment Date 3" xr10:uid="{7BF33E52-DAE1-4371-BBBA-C8991F493960}" cache="NativeTimeline_Appointment_Date" caption="Day" level="3" selectionLevel="0" scrollPosition="2023-06-27T00:00:00"/>
+  <timeline name="Appointment Date 2" xr10:uid="{527740AB-750D-4187-8225-16D51394F21D}" cache="NativeTimeline_Appointment_Date" caption="Month" level="2" selectionLevel="0" scrollPosition="2024-03-10T00:00:00"/>
+  <timeline name="Appointment Date 3" xr10:uid="{7BF33E52-DAE1-4371-BBBA-C8991F493960}" cache="NativeTimeline_Appointment_Date" caption="Day" level="3" selectionLevel="0" scrollPosition="2024-06-27T00:00:00"/>
 </timelines>
 </file>
 
@@ -53640,24 +54828,24 @@
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A4" s="7">
-        <v>92</v>
+        <v>500</v>
       </c>
       <c r="C4" s="7">
-        <v>14</v>
+        <v>56</v>
       </c>
       <c r="E4" s="7"/>
       <c r="F4" s="15">
         <f>(C4/A4)</f>
-        <v>0.15217391304347827</v>
+        <v>0.112</v>
       </c>
       <c r="H4" s="16">
-        <v>9.2934782608695645</v>
+        <v>10.5</v>
       </c>
       <c r="J4" s="7">
         <v>20</v>
       </c>
       <c r="L4" s="7">
-        <v>855</v>
+        <v>5250</v>
       </c>
       <c r="N4" s="7">
         <v>1</v>
@@ -53694,25 +54882,25 @@
         <v>18</v>
       </c>
       <c r="B9" s="7">
-        <v>15</v>
+        <v>101</v>
       </c>
       <c r="D9" s="10" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="E9" s="11">
-        <v>11.5</v>
+        <v>11.44</v>
       </c>
       <c r="G9" s="10" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="H9" s="11">
-        <v>9.2934782608695645</v>
+        <v>11.55952380952381</v>
       </c>
       <c r="J9" s="10" t="s">
         <v>46</v>
       </c>
       <c r="K9" s="11">
-        <v>10.75</v>
+        <v>10.784615384615385</v>
       </c>
     </row>
     <row r="10" spans="1:14" x14ac:dyDescent="0.3">
@@ -53720,25 +54908,25 @@
         <v>11</v>
       </c>
       <c r="B10" s="7">
-        <v>63</v>
+        <v>343</v>
       </c>
       <c r="D10" s="10" t="s">
-        <v>19</v>
+        <v>25</v>
       </c>
       <c r="E10" s="11">
-        <v>11.111111111111111</v>
+        <v>11.348837209302326</v>
       </c>
       <c r="G10" s="10" t="s">
-        <v>31</v>
+        <v>10</v>
       </c>
       <c r="H10" s="11">
-        <v>9.2934782608695645</v>
+        <v>11.546666666666667</v>
       </c>
       <c r="J10" s="10" t="s">
         <v>47</v>
       </c>
       <c r="K10" s="11">
-        <v>9.1304347826086953</v>
+        <v>10.754237288135593</v>
       </c>
     </row>
     <row r="11" spans="1:14" x14ac:dyDescent="0.3">
@@ -53746,19 +54934,25 @@
         <v>22</v>
       </c>
       <c r="B11" s="7">
-        <v>14</v>
+        <v>56</v>
       </c>
       <c r="D11" s="10" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="E11" s="11">
-        <v>10.071428571428571</v>
+        <v>10.95</v>
+      </c>
+      <c r="G11" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="H11" s="11">
+        <v>11.48</v>
       </c>
       <c r="J11" s="10" t="s">
         <v>45</v>
       </c>
       <c r="K11" s="11">
-        <v>8.7741935483870961</v>
+        <v>10.246913580246913</v>
       </c>
     </row>
     <row r="12" spans="1:14" x14ac:dyDescent="0.3">
@@ -53766,33 +54960,45 @@
         <v>31</v>
       </c>
       <c r="B12" s="7">
-        <v>92</v>
+        <v>500</v>
       </c>
       <c r="D12" s="10" t="s">
         <v>23</v>
       </c>
       <c r="E12" s="11">
-        <v>9.0833333333333339</v>
+        <v>10.633333333333333</v>
+      </c>
+      <c r="G12" s="10" t="s">
+        <v>24</v>
+      </c>
+      <c r="H12" s="11">
+        <v>10.49438202247191</v>
       </c>
       <c r="J12" s="10" t="s">
         <v>48</v>
       </c>
       <c r="K12" s="11">
-        <v>8.2142857142857135</v>
+        <v>10.21111111111111</v>
       </c>
     </row>
     <row r="13" spans="1:14" x14ac:dyDescent="0.3">
       <c r="D13" s="10" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="E13" s="11">
-        <v>8.8000000000000007</v>
+        <v>10.512658227848101</v>
+      </c>
+      <c r="G13" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="H13" s="11">
+        <v>9.2934782608695645</v>
       </c>
       <c r="J13" s="10" t="s">
         <v>31</v>
       </c>
       <c r="K13" s="11">
-        <v>9.2934782608695645</v>
+        <v>10.5</v>
       </c>
     </row>
     <row r="14" spans="1:14" x14ac:dyDescent="0.3">
@@ -53800,7 +55006,13 @@
         <v>9</v>
       </c>
       <c r="E14" s="11">
-        <v>8.4642857142857135</v>
+        <v>10.375</v>
+      </c>
+      <c r="G14" s="10" t="s">
+        <v>14</v>
+      </c>
+      <c r="H14" s="11">
+        <v>8.9764705882352942</v>
       </c>
     </row>
     <row r="15" spans="1:14" x14ac:dyDescent="0.3">
@@ -53811,10 +55023,16 @@
         <v>30</v>
       </c>
       <c r="D15" s="10" t="s">
-        <v>26</v>
+        <v>13</v>
       </c>
       <c r="E15" s="11">
-        <v>7.666666666666667</v>
+        <v>9.2727272727272734</v>
+      </c>
+      <c r="G15" s="10" t="s">
+        <v>31</v>
+      </c>
+      <c r="H15" s="11">
+        <v>10.5</v>
       </c>
     </row>
     <row r="16" spans="1:14" x14ac:dyDescent="0.3">
@@ -53822,13 +55040,13 @@
         <v>15</v>
       </c>
       <c r="B16" s="12">
-        <v>282</v>
+        <v>1661</v>
       </c>
       <c r="D16" s="10" t="s">
-        <v>21</v>
+        <v>26</v>
       </c>
       <c r="E16" s="11">
-        <v>4.666666666666667</v>
+        <v>7.7</v>
       </c>
       <c r="J16" s="6" t="s">
         <v>29</v>
@@ -53842,27 +55060,27 @@
         <v>9</v>
       </c>
       <c r="B17" s="12">
-        <v>237</v>
+        <v>1162</v>
       </c>
       <c r="D17" s="10" t="s">
         <v>31</v>
       </c>
       <c r="E17" s="11">
-        <v>9.2934782608695645</v>
+        <v>10.5</v>
       </c>
       <c r="J17" s="10" t="s">
         <v>45</v>
       </c>
       <c r="K17" s="12">
-        <v>272</v>
+        <v>1660</v>
       </c>
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A18" s="10" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="B18" s="12">
-        <v>109</v>
+        <v>657</v>
       </c>
       <c r="G18" s="6" t="s">
         <v>62</v>
@@ -53874,15 +55092,15 @@
         <v>46</v>
       </c>
       <c r="K18" s="12">
-        <v>258</v>
+        <v>1402</v>
       </c>
     </row>
     <row r="19" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A19" s="10" t="s">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="B19" s="12">
-        <v>100</v>
+        <v>638</v>
       </c>
       <c r="G19" s="10" t="s">
         <v>16</v>
@@ -53894,7 +55112,7 @@
         <v>47</v>
       </c>
       <c r="K19" s="12">
-        <v>210</v>
+        <v>1269</v>
       </c>
     </row>
     <row r="20" spans="1:11" x14ac:dyDescent="0.3">
@@ -53902,7 +55120,7 @@
         <v>25</v>
       </c>
       <c r="B20" s="12">
-        <v>46</v>
+        <v>488</v>
       </c>
       <c r="D20" s="6" t="s">
         <v>28</v>
@@ -53911,64 +55129,82 @@
         <v>66</v>
       </c>
       <c r="G20" s="10" t="s">
-        <v>31</v>
+        <v>24</v>
       </c>
       <c r="H20" s="13">
-        <v>0.15217391304347827</v>
+        <v>0.1348314606741573</v>
       </c>
       <c r="J20" s="10" t="s">
         <v>48</v>
       </c>
       <c r="K20" s="12">
-        <v>115</v>
+        <v>919</v>
       </c>
     </row>
     <row r="21" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A21" s="10" t="s">
-        <v>13</v>
+        <v>21</v>
       </c>
       <c r="B21" s="12">
-        <v>44</v>
+        <v>286</v>
       </c>
       <c r="D21" s="10" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="E21" s="13">
-        <v>0.33333333333333331</v>
+        <v>0.14556962025316456</v>
+      </c>
+      <c r="G21" s="10" t="s">
+        <v>20</v>
+      </c>
+      <c r="H21" s="13">
+        <v>0.10714285714285714</v>
       </c>
       <c r="J21" s="10" t="s">
         <v>31</v>
       </c>
       <c r="K21" s="12">
-        <v>855</v>
+        <v>5250</v>
       </c>
     </row>
     <row r="22" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A22" s="10" t="s">
-        <v>26</v>
+        <v>13</v>
       </c>
       <c r="B22" s="12">
-        <v>23</v>
+        <v>204</v>
       </c>
       <c r="D22" s="10" t="s">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="E22" s="13">
-        <v>0.25</v>
+        <v>0.13392857142857142</v>
+      </c>
+      <c r="G22" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="H22" s="13">
+        <v>0.10666666666666667</v>
       </c>
     </row>
     <row r="23" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A23" s="10" t="s">
-        <v>21</v>
+        <v>26</v>
       </c>
       <c r="B23" s="12">
+        <v>154</v>
+      </c>
+      <c r="D23" s="10" t="s">
+        <v>19</v>
+      </c>
+      <c r="E23" s="13">
+        <v>0.11666666666666667</v>
+      </c>
+      <c r="G23" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="D23" s="10" t="s">
-        <v>9</v>
-      </c>
-      <c r="E23" s="13">
-        <v>0.10714285714285714</v>
+      <c r="H23" s="13">
+        <v>0.10588235294117647</v>
       </c>
     </row>
     <row r="24" spans="1:11" x14ac:dyDescent="0.3">
@@ -53976,13 +55212,19 @@
         <v>31</v>
       </c>
       <c r="B24" s="12">
-        <v>855</v>
+        <v>5250</v>
       </c>
       <c r="D24" s="10" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="E24" s="13">
-        <v>8.3333333333333329E-2</v>
+        <v>9.3023255813953487E-2</v>
+      </c>
+      <c r="G24" s="10" t="s">
+        <v>10</v>
+      </c>
+      <c r="H24" s="13">
+        <v>5.3333333333333337E-2</v>
       </c>
       <c r="J24" s="6" t="s">
         <v>55</v>
@@ -53993,30 +55235,36 @@
     </row>
     <row r="25" spans="1:11" x14ac:dyDescent="0.3">
       <c r="D25" s="10" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="E25" s="13">
-        <v>0</v>
+        <v>0.08</v>
+      </c>
+      <c r="G25" s="10" t="s">
+        <v>31</v>
+      </c>
+      <c r="H25" s="13">
+        <v>0.112</v>
       </c>
       <c r="J25" s="10" t="s">
         <v>33</v>
       </c>
       <c r="K25" s="12">
-        <v>9</v>
+        <v>44</v>
       </c>
     </row>
     <row r="26" spans="1:11" x14ac:dyDescent="0.3">
       <c r="D26" s="10" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="E26" s="13">
-        <v>0</v>
+        <v>6.6666666666666666E-2</v>
       </c>
       <c r="J26" s="10" t="s">
         <v>34</v>
       </c>
       <c r="K26" s="12">
-        <v>8</v>
+        <v>37</v>
       </c>
     </row>
     <row r="27" spans="1:11" x14ac:dyDescent="0.3">
@@ -54027,16 +55275,16 @@
         <v>60</v>
       </c>
       <c r="D27" s="10" t="s">
-        <v>21</v>
+        <v>13</v>
       </c>
       <c r="E27" s="13">
-        <v>0</v>
+        <v>4.5454545454545456E-2</v>
       </c>
       <c r="J27" s="10" t="s">
         <v>35</v>
       </c>
       <c r="K27" s="12">
-        <v>10</v>
+        <v>48</v>
       </c>
     </row>
     <row r="28" spans="1:11" x14ac:dyDescent="0.3">
@@ -54044,10 +55292,10 @@
         <v>33</v>
       </c>
       <c r="B28" s="11">
-        <v>7.5555555555555554</v>
+        <v>10.659090909090908</v>
       </c>
       <c r="D28" s="10" t="s">
-        <v>13</v>
+        <v>26</v>
       </c>
       <c r="E28" s="13">
         <v>0</v>
@@ -54062,7 +55310,7 @@
         <v>36</v>
       </c>
       <c r="K28" s="12">
-        <v>7</v>
+        <v>34</v>
       </c>
     </row>
     <row r="29" spans="1:11" x14ac:dyDescent="0.3">
@@ -54070,25 +55318,25 @@
         <v>34</v>
       </c>
       <c r="B29" s="11">
-        <v>8.625</v>
+        <v>10.567567567567568</v>
       </c>
       <c r="D29" s="10" t="s">
         <v>31</v>
       </c>
       <c r="E29" s="13">
-        <v>0.15217391304347827</v>
+        <v>0.112</v>
       </c>
       <c r="G29" s="10" t="s">
         <v>33</v>
       </c>
       <c r="H29" s="13">
-        <v>0</v>
+        <v>9.0909090909090912E-2</v>
       </c>
       <c r="J29" s="10" t="s">
         <v>37</v>
       </c>
       <c r="K29" s="12">
-        <v>3</v>
+        <v>40</v>
       </c>
     </row>
     <row r="30" spans="1:11" x14ac:dyDescent="0.3">
@@ -54096,19 +55344,19 @@
         <v>35</v>
       </c>
       <c r="B30" s="11">
-        <v>11.8</v>
+        <v>11.3125</v>
       </c>
       <c r="G30" s="10" t="s">
         <v>34</v>
       </c>
       <c r="H30" s="13">
-        <v>0.125</v>
+        <v>0.13513513513513514</v>
       </c>
       <c r="J30" s="10" t="s">
         <v>38</v>
       </c>
       <c r="K30" s="12">
-        <v>8</v>
+        <v>47</v>
       </c>
     </row>
     <row r="31" spans="1:11" x14ac:dyDescent="0.3">
@@ -54116,19 +55364,19 @@
         <v>36</v>
       </c>
       <c r="B31" s="11">
-        <v>9</v>
+        <v>9.382352941176471</v>
       </c>
       <c r="G31" s="10" t="s">
         <v>35</v>
       </c>
       <c r="H31" s="13">
-        <v>0</v>
+        <v>8.3333333333333329E-2</v>
       </c>
       <c r="J31" s="10" t="s">
         <v>39</v>
       </c>
       <c r="K31" s="12">
-        <v>7</v>
+        <v>38</v>
       </c>
     </row>
     <row r="32" spans="1:11" x14ac:dyDescent="0.3">
@@ -54136,7 +55384,7 @@
         <v>37</v>
       </c>
       <c r="B32" s="11">
-        <v>15.333333333333334</v>
+        <v>9.8000000000000007</v>
       </c>
       <c r="D32" s="6" t="s">
         <v>62</v>
@@ -54148,13 +55396,13 @@
         <v>36</v>
       </c>
       <c r="H32" s="13">
-        <v>0.14285714285714285</v>
+        <v>0.11764705882352941</v>
       </c>
       <c r="J32" s="10" t="s">
         <v>40</v>
       </c>
       <c r="K32" s="12">
-        <v>8</v>
+        <v>37</v>
       </c>
     </row>
     <row r="33" spans="1:12" x14ac:dyDescent="0.3">
@@ -54162,25 +55410,25 @@
         <v>38</v>
       </c>
       <c r="B33" s="11">
-        <v>10.25</v>
+        <v>12.212765957446809</v>
       </c>
       <c r="D33" s="10" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="E33" s="12">
-        <v>855</v>
+        <v>971</v>
       </c>
       <c r="G33" s="10" t="s">
         <v>37</v>
       </c>
       <c r="H33" s="13">
-        <v>0.66666666666666663</v>
+        <v>0.15</v>
       </c>
       <c r="J33" s="10" t="s">
         <v>41</v>
       </c>
       <c r="K33" s="12">
-        <v>8</v>
+        <v>37</v>
       </c>
     </row>
     <row r="34" spans="1:12" x14ac:dyDescent="0.3">
@@ -54188,25 +55436,25 @@
         <v>39</v>
       </c>
       <c r="B34" s="11">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D34" s="10" t="s">
-        <v>31</v>
+        <v>24</v>
       </c>
       <c r="E34" s="12">
-        <v>855</v>
+        <v>934</v>
       </c>
       <c r="G34" s="10" t="s">
         <v>38</v>
       </c>
       <c r="H34" s="13">
-        <v>0.125</v>
+        <v>8.5106382978723402E-2</v>
       </c>
       <c r="J34" s="10" t="s">
         <v>42</v>
       </c>
       <c r="K34" s="12">
-        <v>7</v>
+        <v>47</v>
       </c>
     </row>
     <row r="35" spans="1:12" x14ac:dyDescent="0.3">
@@ -54214,19 +55462,25 @@
         <v>40</v>
       </c>
       <c r="B35" s="11">
-        <v>10.625</v>
+        <v>9.6486486486486491</v>
+      </c>
+      <c r="D35" s="10" t="s">
+        <v>10</v>
+      </c>
+      <c r="E35" s="12">
+        <v>866</v>
       </c>
       <c r="G35" s="10" t="s">
         <v>39</v>
       </c>
       <c r="H35" s="13">
-        <v>0</v>
+        <v>0.15789473684210525</v>
       </c>
       <c r="J35" s="10" t="s">
         <v>43</v>
       </c>
       <c r="K35" s="12">
-        <v>8</v>
+        <v>52</v>
       </c>
     </row>
     <row r="36" spans="1:12" x14ac:dyDescent="0.3">
@@ -54234,19 +55488,25 @@
         <v>41</v>
       </c>
       <c r="B36" s="11">
-        <v>6.625</v>
+        <v>9.8378378378378386</v>
+      </c>
+      <c r="D36" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="E36" s="12">
+        <v>861</v>
       </c>
       <c r="G36" s="10" t="s">
         <v>40</v>
       </c>
       <c r="H36" s="13">
-        <v>0.125</v>
+        <v>0.13513513513513514</v>
       </c>
       <c r="J36" s="10" t="s">
         <v>44</v>
       </c>
       <c r="K36" s="12">
-        <v>9</v>
+        <v>39</v>
       </c>
     </row>
     <row r="37" spans="1:12" x14ac:dyDescent="0.3">
@@ -54254,19 +55514,25 @@
         <v>42</v>
       </c>
       <c r="B37" s="11">
-        <v>6.8571428571428568</v>
+        <v>10.148936170212766</v>
+      </c>
+      <c r="D37" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="E37" s="12">
+        <v>855</v>
       </c>
       <c r="G37" s="10" t="s">
         <v>41</v>
       </c>
       <c r="H37" s="13">
-        <v>0.375</v>
+        <v>0.21621621621621623</v>
       </c>
       <c r="J37" s="10" t="s">
         <v>31</v>
       </c>
       <c r="K37" s="12">
-        <v>92</v>
+        <v>500</v>
       </c>
     </row>
     <row r="38" spans="1:12" x14ac:dyDescent="0.3">
@@ -54274,13 +55540,19 @@
         <v>43</v>
       </c>
       <c r="B38" s="11">
-        <v>10</v>
+        <v>12.307692307692308</v>
+      </c>
+      <c r="D38" s="10" t="s">
+        <v>14</v>
+      </c>
+      <c r="E38" s="12">
+        <v>763</v>
       </c>
       <c r="G38" s="10" t="s">
         <v>42</v>
       </c>
       <c r="H38" s="13">
-        <v>0.14285714285714285</v>
+        <v>6.3829787234042548E-2</v>
       </c>
       <c r="L38" s="14"/>
     </row>
@@ -54289,13 +55561,19 @@
         <v>44</v>
       </c>
       <c r="B39" s="11">
-        <v>8.1111111111111107</v>
+        <v>9.7948717948717956</v>
+      </c>
+      <c r="D39" s="10" t="s">
+        <v>31</v>
+      </c>
+      <c r="E39" s="12">
+        <v>5250</v>
       </c>
       <c r="G39" s="10" t="s">
         <v>43</v>
       </c>
       <c r="H39" s="13">
-        <v>0.25</v>
+        <v>9.6153846153846159E-2</v>
       </c>
       <c r="L39" s="14"/>
     </row>
@@ -54304,13 +55582,13 @@
         <v>31</v>
       </c>
       <c r="B40" s="11">
-        <v>9.2934782608695645</v>
+        <v>10.5</v>
       </c>
       <c r="G40" s="10" t="s">
         <v>44</v>
       </c>
       <c r="H40" s="13">
-        <v>0.22222222222222221</v>
+        <v>5.128205128205128E-2</v>
       </c>
       <c r="L40" s="14"/>
     </row>
@@ -54319,7 +55597,7 @@
         <v>31</v>
       </c>
       <c r="H41" s="13">
-        <v>0.15217391304347827</v>
+        <v>0.112</v>
       </c>
       <c r="L41" s="14"/>
     </row>
@@ -54334,10 +55612,10 @@
     </row>
     <row r="43" spans="1:12" x14ac:dyDescent="0.3">
       <c r="D43" s="10" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="E43" s="13">
-        <v>0.22580645161290322</v>
+        <v>0.15555555555555556</v>
       </c>
     </row>
     <row r="44" spans="1:12" x14ac:dyDescent="0.3">
@@ -54348,10 +55626,10 @@
         <v>30</v>
       </c>
       <c r="D44" s="10" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="E44" s="13">
-        <v>0.21428571428571427</v>
+        <v>0.1419753086419753</v>
       </c>
     </row>
     <row r="45" spans="1:12" x14ac:dyDescent="0.3">
@@ -54359,13 +55637,13 @@
         <v>33</v>
       </c>
       <c r="B45" s="12">
-        <v>68</v>
+        <v>469</v>
       </c>
       <c r="D45" s="10" t="s">
         <v>46</v>
       </c>
       <c r="E45" s="13">
-        <v>0.125</v>
+        <v>0.1076923076923077</v>
       </c>
     </row>
     <row r="46" spans="1:12" x14ac:dyDescent="0.3">
@@ -54373,13 +55651,13 @@
         <v>34</v>
       </c>
       <c r="B46" s="12">
-        <v>69</v>
+        <v>391</v>
       </c>
       <c r="D46" s="10" t="s">
         <v>47</v>
       </c>
       <c r="E46" s="13">
-        <v>4.3478260869565216E-2</v>
+        <v>4.2372881355932202E-2</v>
       </c>
     </row>
     <row r="47" spans="1:12" x14ac:dyDescent="0.3">
@@ -54387,13 +55665,13 @@
         <v>35</v>
       </c>
       <c r="B47" s="12">
-        <v>118</v>
+        <v>543</v>
       </c>
       <c r="D47" s="10" t="s">
         <v>31</v>
       </c>
       <c r="E47" s="13">
-        <v>0.15217391304347827</v>
+        <v>0.112</v>
       </c>
       <c r="L47" s="9"/>
     </row>
@@ -54402,7 +55680,7 @@
         <v>36</v>
       </c>
       <c r="B48" s="12">
-        <v>63</v>
+        <v>319</v>
       </c>
       <c r="L48" s="14"/>
     </row>
@@ -54411,7 +55689,7 @@
         <v>37</v>
       </c>
       <c r="B49" s="12">
-        <v>46</v>
+        <v>392</v>
       </c>
       <c r="L49" s="14"/>
     </row>
@@ -54420,7 +55698,7 @@
         <v>38</v>
       </c>
       <c r="B50" s="12">
-        <v>82</v>
+        <v>574</v>
       </c>
       <c r="L50" s="14"/>
     </row>
@@ -54429,7 +55707,7 @@
         <v>39</v>
       </c>
       <c r="B51" s="12">
-        <v>70</v>
+        <v>342</v>
       </c>
       <c r="L51" s="14"/>
     </row>
@@ -54438,7 +55716,7 @@
         <v>40</v>
       </c>
       <c r="B52" s="12">
-        <v>85</v>
+        <v>357</v>
       </c>
       <c r="L52" s="14"/>
     </row>
@@ -54447,7 +55725,7 @@
         <v>41</v>
       </c>
       <c r="B53" s="12">
-        <v>53</v>
+        <v>364</v>
       </c>
       <c r="L53" s="14"/>
     </row>
@@ -54456,7 +55734,7 @@
         <v>42</v>
       </c>
       <c r="B54" s="12">
-        <v>48</v>
+        <v>477</v>
       </c>
     </row>
     <row r="55" spans="1:12" x14ac:dyDescent="0.3">
@@ -54464,7 +55742,7 @@
         <v>43</v>
       </c>
       <c r="B55" s="12">
-        <v>80</v>
+        <v>640</v>
       </c>
     </row>
     <row r="56" spans="1:12" x14ac:dyDescent="0.3">
@@ -54472,7 +55750,7 @@
         <v>44</v>
       </c>
       <c r="B56" s="12">
-        <v>73</v>
+        <v>382</v>
       </c>
     </row>
     <row r="57" spans="1:12" x14ac:dyDescent="0.3">
@@ -54480,7 +55758,7 @@
         <v>31</v>
       </c>
       <c r="B57" s="12">
-        <v>855</v>
+        <v>5250</v>
       </c>
     </row>
     <row r="58" spans="1:12" x14ac:dyDescent="0.3">

</xml_diff>